<commit_message>
Updated TestNG setup, fixed Allure reporting, improved registration-login flow
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/TestData.xlsx
+++ b/src/test/resources/TestData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CHANDAN\eclipse-workspace\SeleniumProject\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC6E3A8-F46E-4AB0-A285-FAF642708B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A56266B8-5430-4DAC-A0D2-C55473D0C718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,30 +25,84 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>UserName</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
   <si>
     <t>Password</t>
   </si>
   <si>
-    <t>chans</t>
-  </si>
-  <si>
-    <t>chandus</t>
-  </si>
-  <si>
-    <t>rohits</t>
-  </si>
-  <si>
-    <t>rohitgaut</t>
-  </si>
-  <si>
-    <t>rahuls</t>
-  </si>
-  <si>
-    <t>rahulkuttu</t>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>ZipCode</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>SSN</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>singh</t>
+  </si>
+  <si>
+    <t>hinjewadi</t>
+  </si>
+  <si>
+    <t>pune</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>rajesh</t>
+  </si>
+  <si>
+    <t>brajesh</t>
+  </si>
+  <si>
+    <t>avadhesh</t>
+  </si>
+  <si>
+    <t>santosh</t>
+  </si>
+  <si>
+    <t>rajeshgautu</t>
+  </si>
+  <si>
+    <t>brajeshgautu</t>
+  </si>
+  <si>
+    <t>avadheshgautu</t>
+  </si>
+  <si>
+    <t>santoshgautu</t>
+  </si>
+  <si>
+    <t>GautamRajesh</t>
+  </si>
+  <si>
+    <t>GautamBrajesh</t>
+  </si>
+  <si>
+    <t>GautamAvadhesh</t>
+  </si>
+  <si>
+    <t>GautamSantosh</t>
   </si>
 </sst>
 </file>
@@ -366,43 +420,179 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15.77734375" customWidth="1"/>
+    <col min="8" max="8" width="12.5546875" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" customWidth="1"/>
+    <col min="10" max="10" width="14.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2">
+        <v>412106</v>
+      </c>
+      <c r="G2">
+        <v>9960674335</v>
+      </c>
+      <c r="H2">
+        <v>12345678</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3">
+        <v>412106</v>
+      </c>
+      <c r="G3">
+        <v>9006105733</v>
+      </c>
+      <c r="H3">
+        <v>12345678</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4">
+        <v>412106</v>
+      </c>
+      <c r="G4">
+        <v>9631692459</v>
+      </c>
+      <c r="H4">
+        <v>12345678</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5">
+        <v>412106</v>
+      </c>
+      <c r="G5">
+        <v>9970436666</v>
+      </c>
+      <c r="H5">
+        <v>12345678</v>
+      </c>
+      <c r="I5" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>